<commit_message>
CNG commit CngPages Final commit
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/CngCarsRatingGreaterThan_4.xlsx
+++ b/src/test/resources/testData/CngCarsRatingGreaterThan_4.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Car Name</t>
   </si>
@@ -32,61 +32,37 @@
     <t>Maruti Suzuki Ertiga</t>
   </si>
   <si>
+    <t>Maruti Suzuki Swift</t>
+  </si>
+  <si>
     <t>Maruti Suzuki Brezza</t>
   </si>
   <si>
+    <t>Maruti Suzuki Baleno</t>
+  </si>
+  <si>
     <t>Maruti Suzuki Dzire</t>
   </si>
   <si>
     <t>Hyundai Aura</t>
   </si>
   <si>
+    <t>Toyota Urban Cruiser Hyryder</t>
+  </si>
+  <si>
+    <t>Nissan Gravite</t>
+  </si>
+  <si>
     <t>Tata Tiago</t>
   </si>
   <si>
+    <t>Kia Carens</t>
+  </si>
+  <si>
     <t>Hyundai Exter</t>
   </si>
   <si>
-    <t>Kia Carens</t>
-  </si>
-  <si>
-    <t>Maruti Suzuki Victoris</t>
-  </si>
-  <si>
-    <t>Tata Altroz</t>
-  </si>
-  <si>
-    <t>Citroen C3</t>
-  </si>
-  <si>
-    <t>Nissan Magnite</t>
-  </si>
-  <si>
-    <t>Toyota Rumion</t>
-  </si>
-  <si>
-    <t>Maruti Suzuki XL6</t>
-  </si>
-  <si>
-    <t>Bajaj Qute</t>
-  </si>
-  <si>
-    <t>Tata Xpres</t>
-  </si>
-  <si>
-    <t>Maruti Suzuki Dzire Tour S</t>
-  </si>
-  <si>
-    <t>Hyundai Prime SD</t>
-  </si>
-  <si>
-    <t>Maruti Suzuki Ertiga Tour</t>
-  </si>
-  <si>
-    <t>Maruti Suzuki Grand Vitara</t>
-  </si>
-  <si>
-    <t>Maruti Suzuki Eeco Cargo</t>
+    <t>Maruti Suzuki Wagon R</t>
   </si>
 </sst>
 </file>
@@ -131,7 +107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -187,7 +163,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="8">
@@ -203,7 +179,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="10">
@@ -211,7 +187,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="n" s="0">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="11">
@@ -219,7 +195,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="n" s="0">
-        <v>5.0</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="12">
@@ -227,7 +203,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="n" s="0">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="13">
@@ -235,7 +211,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="n" s="0">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="14">
@@ -243,7 +219,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="15">
@@ -259,70 +235,6 @@
         <v>16</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="B17" t="n" s="0">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B18" t="n" s="0">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="B19" t="n" s="0">
-        <v>4.7</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="B20" t="n" s="0">
-        <v>4.1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="B21" t="n" s="0">
-        <v>4.4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B22" t="n" s="0">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="B23" t="n" s="0">
-        <v>4.4</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="B24" t="n" s="0">
         <v>4.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CNG commit CngPages price xpath
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/CngCarsRatingGreaterThan_4.xlsx
+++ b/src/test/resources/testData/CngCarsRatingGreaterThan_4.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Car Name</t>
   </si>
@@ -56,13 +56,16 @@
     <t>Tata Tiago</t>
   </si>
   <si>
-    <t>Kia Carens</t>
-  </si>
-  <si>
-    <t>Hyundai Exter</t>
-  </si>
-  <si>
     <t>Maruti Suzuki Wagon R</t>
+  </si>
+  <si>
+    <t>Maruti Suzuki Alto K10</t>
+  </si>
+  <si>
+    <t>Maruti Suzuki Victoris</t>
+  </si>
+  <si>
+    <t>Tata Altroz</t>
   </si>
 </sst>
 </file>
@@ -107,7 +110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -219,7 +222,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>4.6</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="15">
@@ -227,7 +230,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="n" s="0">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="16">
@@ -235,6 +238,14 @@
         <v>16</v>
       </c>
       <c r="B16" t="n" s="0">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B17" t="n" s="0">
         <v>4.4</v>
       </c>
     </row>

</xml_diff>